<commit_message>
Add Middle Earth TMDB Posters
</commit_message>
<xml_diff>
--- a/MIDDLEEARTH.xlsx
+++ b/MIDDLEEARTH.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="MIDDLEEARTH" sheetId="1" state="visible" r:id="rId1"/>
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="19">
+  <fonts count="2">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -27,319 +27,21 @@
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <color theme="1"/>
+      <color theme="10"/>
       <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Display"/>
-      <family val="2"/>
-      <color theme="3"/>
-      <sz val="18"/>
-      <scheme val="major"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="15"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="13"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <color rgb="FF006100"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <color rgb="FF9C0006"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <color rgb="FF9C5700"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <color rgb="FF3F3F76"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF3F3F3F"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color rgb="FFFA7D00"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <color rgb="FFFA7D00"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color theme="0"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <color rgb="FFFF0000"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <i val="1"/>
-      <color rgb="FF7F7F7F"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <color theme="0"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <sz val="8"/>
+      <u val="single"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.7999816888943144"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.5999938962981048"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.3999755851924192"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.7999816888943144"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.5999938962981048"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.3999755851924192"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.7999816888943144"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.5999938962981048"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.3999755851924192"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.7999816888943144"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.5999938962981048"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.3999755851924192"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.7999816888943144"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.5999938962981048"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.3999755851924192"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.7999816888943144"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.5999938962981048"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.3999755851924192"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="10">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -347,205 +49,19 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thick">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thick">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.3999755851924192"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="42">
+  <cellStyleXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="4"/>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="5"/>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="4"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6"/>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="7"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="8"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9"/>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="15" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="16" borderId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="17" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="18" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="20" borderId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="21" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="22" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="23" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="24" borderId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="25" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="26" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="27" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="28" borderId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="29" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="30" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="31" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="32" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="42">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Title" xfId="1" builtinId="15"/>
-    <cellStyle name="Heading 1" xfId="2" builtinId="16"/>
-    <cellStyle name="Heading 2" xfId="3" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="4" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="5" builtinId="19"/>
-    <cellStyle name="Good" xfId="6" builtinId="26"/>
-    <cellStyle name="Bad" xfId="7" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="8" builtinId="28"/>
-    <cellStyle name="Input" xfId="9" builtinId="20"/>
-    <cellStyle name="Output" xfId="10" builtinId="21"/>
-    <cellStyle name="Calculation" xfId="11" builtinId="22"/>
-    <cellStyle name="Linked Cell" xfId="12" builtinId="24"/>
-    <cellStyle name="Check Cell" xfId="13" builtinId="23"/>
-    <cellStyle name="Warning Text" xfId="14" builtinId="11"/>
-    <cellStyle name="Note" xfId="15" builtinId="10"/>
-    <cellStyle name="Explanatory Text" xfId="16" builtinId="53"/>
-    <cellStyle name="Total" xfId="17" builtinId="25"/>
-    <cellStyle name="Accent1" xfId="18" builtinId="29"/>
-    <cellStyle name="20% - Accent1" xfId="19" builtinId="30"/>
-    <cellStyle name="40% - Accent1" xfId="20" builtinId="31"/>
-    <cellStyle name="60% - Accent1" xfId="21" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="22" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="23" builtinId="34"/>
-    <cellStyle name="40% - Accent2" xfId="24" builtinId="35"/>
-    <cellStyle name="60% - Accent2" xfId="25" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="26" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="27" builtinId="38"/>
-    <cellStyle name="40% - Accent3" xfId="28" builtinId="39"/>
-    <cellStyle name="60% - Accent3" xfId="29" builtinId="40"/>
-    <cellStyle name="Accent4" xfId="30" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="31" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="32" builtinId="43"/>
-    <cellStyle name="60% - Accent4" xfId="33" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="34" builtinId="45"/>
-    <cellStyle name="20% - Accent5" xfId="35" builtinId="46"/>
-    <cellStyle name="40% - Accent5" xfId="36" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="37" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="38" builtinId="49"/>
-    <cellStyle name="20% - Accent6" xfId="39" builtinId="50"/>
-    <cellStyle name="40% - Accent6" xfId="40" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="41" builtinId="52"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -950,6 +466,7 @@
     <col width="15" customWidth="1" min="10" max="10"/>
     <col width="50.28515625" customWidth="1" min="11" max="11"/>
     <col width="72.28515625" customWidth="1" min="12" max="12"/>
+    <col width="51.140625" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1059,11 +576,6 @@
           <t>Middle Earth</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>the-silmarillion.jpg</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1095,11 +607,6 @@
           <t>Middle Earth</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>the-children-of-hurin.jpg</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1131,11 +638,6 @@
           <t>Middle Earth</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>beren-and-luthien.jpg</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1167,11 +669,6 @@
           <t>Middle Earth</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>the-fall-of-gondolin.jpg</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1203,11 +700,6 @@
           <t>Middle Earth</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>unfinished-tales-of-numenor-and-middle-earth.jpg</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1254,12 +746,22 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>the-lord-of-the-rings-the-rings-of-power-s1.jpg</t>
+          <t>https://image.tmdb.org/t/p/w500/zZVQbQV7djOnO8ugeJ8iQKm3I4U.jpg</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt9788618/?ref_=ttep_ep_1</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/tv/84773-the-lord-of-the-rings-the-rings-of-power/season/1</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>tv</t>
         </is>
       </c>
     </row>
@@ -1308,12 +810,22 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>the-lord-of-the-rings-the-rings-of-power-s1.jpg</t>
+          <t>https://image.tmdb.org/t/p/w500/zZVQbQV7djOnO8ugeJ8iQKm3I4U.jpg</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt10582302/?ref_=ttep_ep_2</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/tv/84773-the-lord-of-the-rings-the-rings-of-power/season/1</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>tv</t>
         </is>
       </c>
     </row>
@@ -1362,12 +874,22 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>the-lord-of-the-rings-the-rings-of-power-s1.jpg</t>
+          <t>https://image.tmdb.org/t/p/w500/zZVQbQV7djOnO8ugeJ8iQKm3I4U.jpg</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt11609034/?ref_=ttep_ep_3</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/tv/84773-the-lord-of-the-rings-the-rings-of-power/season/1</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>tv</t>
         </is>
       </c>
     </row>
@@ -1416,12 +938,22 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>the-lord-of-the-rings-the-rings-of-power-s1.jpg</t>
+          <t>https://image.tmdb.org/t/p/w500/zZVQbQV7djOnO8ugeJ8iQKm3I4U.jpg</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt11609038/?ref_=ttep_ep_4</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/tv/84773-the-lord-of-the-rings-the-rings-of-power/season/1</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>tv</t>
         </is>
       </c>
     </row>
@@ -1470,12 +1002,22 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>the-lord-of-the-rings-the-rings-of-power-s1.jpg</t>
+          <t>https://image.tmdb.org/t/p/w500/zZVQbQV7djOnO8ugeJ8iQKm3I4U.jpg</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt11609040/?ref_=ttep_ep_5</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/tv/84773-the-lord-of-the-rings-the-rings-of-power/season/1</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>tv</t>
         </is>
       </c>
     </row>
@@ -1524,12 +1066,22 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>the-lord-of-the-rings-the-rings-of-power-s1.jpg</t>
+          <t>https://image.tmdb.org/t/p/w500/zZVQbQV7djOnO8ugeJ8iQKm3I4U.jpg</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt11609042/?ref_=ttep_ep_6</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/tv/84773-the-lord-of-the-rings-the-rings-of-power/season/1</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>tv</t>
         </is>
       </c>
     </row>
@@ -1578,12 +1130,22 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>the-lord-of-the-rings-the-rings-of-power-s1.jpg</t>
+          <t>https://image.tmdb.org/t/p/w500/zZVQbQV7djOnO8ugeJ8iQKm3I4U.jpg</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt11609046/?ref_=ttep_ep_7</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/tv/84773-the-lord-of-the-rings-the-rings-of-power/season/1</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>tv</t>
         </is>
       </c>
     </row>
@@ -1632,12 +1194,22 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>the-lord-of-the-rings-the-rings-of-power-s1.jpg</t>
+          <t>https://image.tmdb.org/t/p/w500/zZVQbQV7djOnO8ugeJ8iQKm3I4U.jpg</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt11609048/?ref_=ttep_ep_8</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/tv/84773-the-lord-of-the-rings-the-rings-of-power/season/1</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>tv</t>
         </is>
       </c>
     </row>
@@ -1686,12 +1258,22 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>the-lord-of-the-rings-the-rings-of-power-s2.jpg</t>
+          <t>https://image.tmdb.org/t/p/w500/eTQLv1sjLhDBPwI2u0qaqV51HWU.jpg</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt13580784/?ref_=ttep_ep_1</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/tv/84773-the-lord-of-the-rings-the-rings-of-power/season/2</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>tv</t>
         </is>
       </c>
     </row>
@@ -1740,12 +1322,22 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>the-lord-of-the-rings-the-rings-of-power-s2.jpg</t>
+          <t>https://image.tmdb.org/t/p/w500/eTQLv1sjLhDBPwI2u0qaqV51HWU.jpg</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt27580486/?ref_=ttep_ep_2</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/tv/84773-the-lord-of-the-rings-the-rings-of-power/season/2</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>tv</t>
         </is>
       </c>
     </row>
@@ -1794,12 +1386,22 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>the-lord-of-the-rings-the-rings-of-power-s2.jpg</t>
+          <t>https://image.tmdb.org/t/p/w500/eTQLv1sjLhDBPwI2u0qaqV51HWU.jpg</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt27580490/?ref_=ttep_ep_3</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/tv/84773-the-lord-of-the-rings-the-rings-of-power/season/2</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>tv</t>
         </is>
       </c>
     </row>
@@ -1848,12 +1450,22 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>the-lord-of-the-rings-the-rings-of-power-s2.jpg</t>
+          <t>https://image.tmdb.org/t/p/w500/eTQLv1sjLhDBPwI2u0qaqV51HWU.jpg</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt27580491/?ref_=ttep_ep_4</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/tv/84773-the-lord-of-the-rings-the-rings-of-power/season/2</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>tv</t>
         </is>
       </c>
     </row>
@@ -1902,12 +1514,22 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>the-lord-of-the-rings-the-rings-of-power-s2.jpg</t>
+          <t>https://image.tmdb.org/t/p/w500/eTQLv1sjLhDBPwI2u0qaqV51HWU.jpg</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt27580494/?ref_=ttep_ep_5</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/tv/84773-the-lord-of-the-rings-the-rings-of-power/season/2</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>tv</t>
         </is>
       </c>
     </row>
@@ -1956,12 +1578,22 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>the-lord-of-the-rings-the-rings-of-power-s2.jpg</t>
+          <t>https://image.tmdb.org/t/p/w500/eTQLv1sjLhDBPwI2u0qaqV51HWU.jpg</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt27580495/?ref_=ttep_ep_6</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/tv/84773-the-lord-of-the-rings-the-rings-of-power/season/2</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>tv</t>
         </is>
       </c>
     </row>
@@ -2010,12 +1642,22 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>the-lord-of-the-rings-the-rings-of-power-s2.jpg</t>
+          <t>https://image.tmdb.org/t/p/w500/eTQLv1sjLhDBPwI2u0qaqV51HWU.jpg</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt27580496/?ref_=ttep_ep_7</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/tv/84773-the-lord-of-the-rings-the-rings-of-power/season/2</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>tv</t>
         </is>
       </c>
     </row>
@@ -2064,12 +1706,22 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>the-lord-of-the-rings-the-rings-of-power-s2.jpg</t>
+          <t>https://image.tmdb.org/t/p/w500/eTQLv1sjLhDBPwI2u0qaqV51HWU.jpg</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt27580497/?ref_=ttep_ep_8</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/tv/84773-the-lord-of-the-rings-the-rings-of-power/season/2</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>tv</t>
         </is>
       </c>
     </row>
@@ -2110,12 +1762,22 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>the-lord-of-the-rings-the-rings-of-power-s3.jpg</t>
+          <t>https://image.tmdb.org/t/p/w500/xw9VIpdX0n0BNQRMLWj8Y0T4yew.jpg</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt32446124/?ref_=ttep_ep_1</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/tv/84773-the-lord-of-the-rings-the-rings-of-power/season/3</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>tv</t>
         </is>
       </c>
     </row>
@@ -2156,12 +1818,22 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>the-lord-of-the-rings-the-rings-of-power-s3.jpg</t>
+          <t>https://image.tmdb.org/t/p/w500/xw9VIpdX0n0BNQRMLWj8Y0T4yew.jpg</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt41902171/?ref_=ttep_ep_2</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/tv/84773-the-lord-of-the-rings-the-rings-of-power/season/3</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>tv</t>
         </is>
       </c>
     </row>
@@ -2202,12 +1874,22 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>the-lord-of-the-rings-the-rings-of-power-s3.jpg</t>
+          <t>https://image.tmdb.org/t/p/w500/xw9VIpdX0n0BNQRMLWj8Y0T4yew.jpg</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt41902174/?ref_=ttep_ep_3</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/tv/84773-the-lord-of-the-rings-the-rings-of-power/season/3</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>tv</t>
         </is>
       </c>
     </row>
@@ -2248,12 +1930,22 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>the-lord-of-the-rings-the-rings-of-power-s3.jpg</t>
+          <t>https://image.tmdb.org/t/p/w500/xw9VIpdX0n0BNQRMLWj8Y0T4yew.jpg</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt41902181/?ref_=ttep_ep_4</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/tv/84773-the-lord-of-the-rings-the-rings-of-power/season/3</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>tv</t>
         </is>
       </c>
     </row>
@@ -2294,12 +1986,22 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>the-lord-of-the-rings-the-rings-of-power-s3.jpg</t>
+          <t>https://image.tmdb.org/t/p/w500/xw9VIpdX0n0BNQRMLWj8Y0T4yew.jpg</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt41902190/?ref_=ttep_ep_5</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/tv/84773-the-lord-of-the-rings-the-rings-of-power/season/3</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>tv</t>
         </is>
       </c>
     </row>
@@ -2340,12 +2042,22 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>the-lord-of-the-rings-the-rings-of-power-s3.jpg</t>
+          <t>https://image.tmdb.org/t/p/w500/xw9VIpdX0n0BNQRMLWj8Y0T4yew.jpg</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt41902191/?ref_=ttep_ep_6</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/tv/84773-the-lord-of-the-rings-the-rings-of-power/season/3</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>tv</t>
         </is>
       </c>
     </row>
@@ -2386,12 +2098,22 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>the-lord-of-the-rings-the-rings-of-power-s3.jpg</t>
+          <t>https://image.tmdb.org/t/p/w500/xw9VIpdX0n0BNQRMLWj8Y0T4yew.jpg</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt41902195/?ref_=ttep_ep_7</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/tv/84773-the-lord-of-the-rings-the-rings-of-power/season/3</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>tv</t>
         </is>
       </c>
     </row>
@@ -2432,12 +2154,22 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>the-lord-of-the-rings-the-rings-of-power-s3.jpg</t>
+          <t>https://image.tmdb.org/t/p/w500/xw9VIpdX0n0BNQRMLWj8Y0T4yew.jpg</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt41902197/?ref_=ttep_ep_8</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/tv/84773-the-lord-of-the-rings-the-rings-of-power/season/3</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>tv</t>
         </is>
       </c>
     </row>
@@ -2476,7 +2208,7 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>the-lord-of-the-rings-the-war-of-the-rohirrim.jpg</t>
+          <t>https://image.tmdb.org/t/p/w500/23WCoDo6wzBfzbX7BGTNwVUqZfi.jpg</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
@@ -2487,6 +2219,16 @@
       <c r="M31" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt14824600/</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/movie/839033-the-lord-of-the-rings-the-war-of-the-rohirrim</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>movie</t>
         </is>
       </c>
     </row>
@@ -2520,11 +2262,6 @@
           <t>Middle Earth</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>the-hobbit-or-there-and-back-again.jpg</t>
-        </is>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2561,7 +2298,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>the-hobbit.jpg</t>
+          <t>https://image.tmdb.org/t/p/w500/2ohvyMPhvjftLrM6S6Ljr6QrL0u.jpg</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
@@ -2572,6 +2309,16 @@
       <c r="M33" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt0077687/</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/movie/1362-the-hobbit</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>movie</t>
         </is>
       </c>
     </row>
@@ -2610,7 +2357,7 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>the-hobbit-an-unexpected-journey.jpg</t>
+          <t>https://image.tmdb.org/t/p/w500/yHA9Fc37VmpUA5UncTxxo3rTGVA.jpg</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
@@ -2621,6 +2368,16 @@
       <c r="M34" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt0903624/</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/movie/49051-the-hobbit-an-unexpected-journey</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>movie</t>
         </is>
       </c>
     </row>
@@ -2659,7 +2416,7 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>the-hobbit-the-desolation-of-smaug.jpg</t>
+          <t>https://image.tmdb.org/t/p/w500/xQYiXsheRCDBA39DOrmaw1aSpbk.jpg</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
@@ -2670,6 +2427,16 @@
       <c r="M35" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt1170358/</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/movie/57158-the-hobbit-the-desolation-of-smaug</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>movie</t>
         </is>
       </c>
     </row>
@@ -2708,7 +2475,7 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>the-hobbit-the-battle-of-the-five-armies.jpg</t>
+          <t>https://image.tmdb.org/t/p/w500/xT98tLqatZPQApyRmlPL12LtiWp.jpg</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
@@ -2719,6 +2486,16 @@
       <c r="M36" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt2310332/</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/movie/122917-the-hobbit-the-battle-of-the-five-armies</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>movie</t>
         </is>
       </c>
     </row>
@@ -2752,11 +2529,6 @@
           <t>Middle Earth</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>tales-of-the-shire.jpg</t>
-        </is>
-      </c>
       <c r="M37" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt32650767/</t>
@@ -2793,11 +2565,6 @@
           <t>Middle Earth</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>shadow-of-mordor.jpg</t>
-        </is>
-      </c>
       <c r="M38" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt3330488/</t>
@@ -2834,11 +2601,6 @@
           <t>Middle Earth</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>shadow-of-war.jpg</t>
-        </is>
-      </c>
       <c r="M39" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt6579422/</t>
@@ -2875,11 +2637,6 @@
           <t>Middle Earth</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>gollum.jpg</t>
-        </is>
-      </c>
       <c r="M40" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt12789698/</t>
@@ -2918,7 +2675,7 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>the-lord-of-the-rings-the-hunt-for-gollum.jpg</t>
+          <t>https://image.tmdb.org/t/p/w500/aRtIVdlgVNtvcqFUnuhR3V1RQ7o.jpg</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
@@ -2929,6 +2686,16 @@
       <c r="M41" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt32328070/</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/movie/1090869-the-lord-of-the-rings-the-hunt-for-gollum</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>movie</t>
         </is>
       </c>
     </row>
@@ -2962,11 +2729,6 @@
           <t>Middle Earth</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>the-fellowship-of-the-ring.jpg</t>
-        </is>
-      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3003,7 +2765,7 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>the-lord-of-the-rings-the-fellowship-of-the-ring.jpg</t>
+          <t>https://image.tmdb.org/t/p/w500/6oom5QYQ2yQTMJIbnvbkBL9cHo6.jpg</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
@@ -3014,6 +2776,16 @@
       <c r="M43" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt0120737/</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/movie/120-the-lord-of-the-rings-the-fellowship-of-the-ring</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>movie</t>
         </is>
       </c>
     </row>
@@ -3047,11 +2819,6 @@
           <t>Middle Earth</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>the-two-towers.jpg</t>
-        </is>
-      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3088,7 +2855,7 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>the-lord-of-the-rings.jpg</t>
+          <t>https://image.tmdb.org/t/p/w500/liW0mjvTyLs7UCumaHhx3PpU4VT.jpg</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
@@ -3099,6 +2866,16 @@
       <c r="M45" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt0077869/</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/movie/123-the-lord-of-the-rings</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>movie</t>
         </is>
       </c>
     </row>
@@ -3137,7 +2914,7 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>the-lord-of-the-rings-the-two-towers.jpg</t>
+          <t>https://image.tmdb.org/t/p/w500/5VTN0pR8gcqV3EPUHHfMGnJYN9L.jpg</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
@@ -3148,6 +2925,16 @@
       <c r="M46" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt0167261/</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/movie/121-the-lord-of-the-rings-the-two-towers</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>movie</t>
         </is>
       </c>
     </row>
@@ -3181,11 +2968,6 @@
           <t>Middle Earth</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>the-return-of-the-king.jpg</t>
-        </is>
-      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3237,7 +3019,7 @@
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>1361-the-return-of-the-king</t>
+          <t>https://www.themoviedb.org/movie/1361-the-return-of-the-king</t>
         </is>
       </c>
       <c r="O48" t="inlineStr">
@@ -3281,7 +3063,7 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>the-lord-of-the-rings-the-return-of-the-king.jpg</t>
+          <t>https://image.tmdb.org/t/p/w500/rCzpDGLbOoPwLjy3OAm5NUPOTrC.jpg</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
@@ -3292,6 +3074,16 @@
       <c r="M49" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt0167260/</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>https://www.themoviedb.org/movie/122-the-lord-of-the-rings-the-return-of-the-king</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>movie</t>
         </is>
       </c>
     </row>
@@ -3325,11 +3117,6 @@
           <t>Middle Earth</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>the-battle-for-middle-earth.jpg</t>
-        </is>
-      </c>
       <c r="M50" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt0412935/</t>
@@ -3366,11 +3153,6 @@
           <t>Middle Earth</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>the-battle-for-middle-earth-ii.jpg</t>
-        </is>
-      </c>
       <c r="M51" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt0760172/</t>
@@ -3407,11 +3189,6 @@
           <t>Middle Earth</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>war-in-the-north.jpg</t>
-        </is>
-      </c>
       <c r="M52" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt2102446/</t>
@@ -3448,11 +3225,6 @@
           <t>Middle Earth</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>return-to-moria.jpg</t>
-        </is>
-      </c>
       <c r="M53" t="inlineStr">
         <is>
           <t>https://www.imdb.com/title/tt29865856/</t>
@@ -3460,6 +3232,9 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Improved Load times and Helstrom added
</commit_message>
<xml_diff>
--- a/MIDDLEEARTH.xlsx
+++ b/MIDDLEEARTH.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benja\timeline-site\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DC70DE5-04F7-4FF5-908D-B513998C3CC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{348B975D-3248-4B7E-89C3-B644A82B1652}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -724,31 +724,31 @@
     <t>https://www.imdb.com/title/tt29865856/</t>
   </si>
   <si>
-    <t>https://covers.openlibrary.org/b/id/10721368-M.jpg</t>
-  </si>
-  <si>
-    <t>https://covers.openlibrary.org/b/id/395259-M.jpg</t>
-  </si>
-  <si>
-    <t>https://covers.openlibrary.org/b/id/12639912-M.jpg</t>
-  </si>
-  <si>
-    <t>https://covers.openlibrary.org/b/id/12451486-M.jpg</t>
-  </si>
-  <si>
-    <t>https://covers.openlibrary.org/b/id/13197860-M.jpg</t>
-  </si>
-  <si>
-    <t>https://covers.openlibrary.org/b/id/15244617-M.jpg</t>
-  </si>
-  <si>
-    <t>https://covers.openlibrary.org/b/id/14844407-M.jpg</t>
-  </si>
-  <si>
-    <t>https://covers.openlibrary.org/b/id/15101803-M.jpg</t>
-  </si>
-  <si>
-    <t>https://covers.openlibrary.org/b/id/15246805-M.jpg</t>
+    <t>https://covers.openlibrary.org/b/id/10721368-L.jpg</t>
+  </si>
+  <si>
+    <t>https://covers.openlibrary.org/b/id/395259-L.jpg</t>
+  </si>
+  <si>
+    <t>https://covers.openlibrary.org/b/id/12639912-L.jpg</t>
+  </si>
+  <si>
+    <t>https://covers.openlibrary.org/b/id/12451486-L.jpg</t>
+  </si>
+  <si>
+    <t>https://covers.openlibrary.org/b/id/13197860-L.jpg</t>
+  </si>
+  <si>
+    <t>https://covers.openlibrary.org/b/id/15244617-L.jpg</t>
+  </si>
+  <si>
+    <t>https://covers.openlibrary.org/b/id/14844407-L.jpg</t>
+  </si>
+  <si>
+    <t>https://covers.openlibrary.org/b/id/15101803-L.jpg</t>
+  </si>
+  <si>
+    <t>https://covers.openlibrary.org/b/id/15246805-L.jpg</t>
   </si>
 </sst>
 </file>
@@ -1133,19 +1133,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P53"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="22.42578125" customWidth="1"/>
-    <col min="4" max="4" width="67.7109375" customWidth="1"/>
-    <col min="6" max="6" width="25.85546875" customWidth="1"/>
-    <col min="7" max="7" width="17.85546875" customWidth="1"/>
+    <col min="1" max="1" width="22.3984375" customWidth="1"/>
+    <col min="4" max="4" width="67.73046875" customWidth="1"/>
+    <col min="6" max="6" width="25.86328125" customWidth="1"/>
+    <col min="7" max="7" width="17.86328125" customWidth="1"/>
     <col min="10" max="10" width="15" customWidth="1"/>
-    <col min="11" max="11" width="50.28515625" customWidth="1"/>
-    <col min="12" max="12" width="72.28515625" customWidth="1"/>
-    <col min="13" max="13" width="51.140625" customWidth="1"/>
+    <col min="11" max="11" width="50.265625" customWidth="1"/>
+    <col min="12" max="12" width="72.265625" customWidth="1"/>
+    <col min="13" max="13" width="51.1328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1195,7 +1195,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -1224,7 +1224,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -1253,7 +1253,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>24</v>
       </c>
@@ -1282,7 +1282,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -1311,7 +1311,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>30</v>
       </c>
@@ -1340,7 +1340,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>33</v>
       </c>
@@ -1384,7 +1384,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>42</v>
       </c>
@@ -1428,7 +1428,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>46</v>
       </c>
@@ -1472,7 +1472,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>50</v>
       </c>
@@ -1516,7 +1516,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>54</v>
       </c>
@@ -1560,7 +1560,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>58</v>
       </c>
@@ -1604,7 +1604,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>62</v>
       </c>
@@ -1648,7 +1648,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>66</v>
       </c>
@@ -1692,7 +1692,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>70</v>
       </c>
@@ -1736,7 +1736,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>76</v>
       </c>
@@ -1780,7 +1780,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>80</v>
       </c>
@@ -1824,7 +1824,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>84</v>
       </c>
@@ -1868,7 +1868,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>88</v>
       </c>
@@ -1912,7 +1912,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>92</v>
       </c>
@@ -1956,7 +1956,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>96</v>
       </c>
@@ -2000,7 +2000,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>100</v>
       </c>
@@ -2044,7 +2044,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>104</v>
       </c>
@@ -2082,7 +2082,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>109</v>
       </c>
@@ -2120,7 +2120,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>112</v>
       </c>
@@ -2158,7 +2158,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>115</v>
       </c>
@@ -2196,7 +2196,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>118</v>
       </c>
@@ -2234,7 +2234,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
         <v>121</v>
       </c>
@@ -2272,7 +2272,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
         <v>124</v>
       </c>
@@ -2310,7 +2310,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
         <v>127</v>
       </c>
@@ -2348,7 +2348,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
         <v>130</v>
       </c>
@@ -2389,7 +2389,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
         <v>138</v>
       </c>
@@ -2418,7 +2418,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
         <v>141</v>
       </c>
@@ -2459,7 +2459,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
         <v>147</v>
       </c>
@@ -2500,7 +2500,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
         <v>153</v>
       </c>
@@ -2541,7 +2541,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
         <v>159</v>
       </c>
@@ -2582,7 +2582,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
         <v>165</v>
       </c>
@@ -2608,7 +2608,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
         <v>169</v>
       </c>
@@ -2634,7 +2634,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
         <v>172</v>
       </c>
@@ -2660,7 +2660,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
         <v>175</v>
       </c>
@@ -2686,7 +2686,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
         <v>178</v>
       </c>
@@ -2724,7 +2724,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
         <v>184</v>
       </c>
@@ -2753,7 +2753,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
         <v>187</v>
       </c>
@@ -2794,7 +2794,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
         <v>193</v>
       </c>
@@ -2823,7 +2823,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
         <v>196</v>
       </c>
@@ -2864,7 +2864,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
         <v>202</v>
       </c>
@@ -2905,7 +2905,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
         <v>208</v>
       </c>
@@ -2934,7 +2934,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
         <v>211</v>
       </c>
@@ -2975,7 +2975,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
         <v>216</v>
       </c>
@@ -3016,7 +3016,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
         <v>222</v>
       </c>
@@ -3042,7 +3042,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
         <v>225</v>
       </c>
@@ -3068,7 +3068,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A52" t="s">
         <v>228</v>
       </c>
@@ -3094,7 +3094,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A53" t="s">
         <v>231</v>
       </c>
@@ -3124,7 +3124,7 @@
   <hyperlinks>
     <hyperlink ref="N16" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="P44" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="K2" r:id="rId3" xr:uid="{223B0864-F33B-4A9F-97F3-B9686705CAFD}"/>
+    <hyperlink ref="K2" r:id="rId3" display="https://covers.openlibrary.org/b/id/10721368-M.jpg" xr:uid="{223B0864-F33B-4A9F-97F3-B9686705CAFD}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>